<commit_message>
Move login/credentials test cases to separate Login folder (46 tests)
</commit_message>
<xml_diff>
--- a/User_Module/Users_Module_Test_Script.xlsx
+++ b/User_Module/Users_Module_Test_Script.xlsx
@@ -86,7 +86,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -107,6 +107,12 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -473,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H75"/>
+  <dimension ref="A1:H76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1705,7 +1711,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>USR_031</t>
+          <t>USR_048</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1715,1819 +1721,1030 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Credentials - Region Selection</t>
+          <t>User Details - Open Panel</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>App launched, credentials screen displayed</t>
+          <t>User conversation selected</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Verify US region is selected by default</t>
+          <t>Verify user details panel opens on header click</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>1. Open app
-2. Navigate to credentials screen
-3. Observe region selector</t>
-        </is>
-      </c>
-      <c r="G33" s="2" t="inlineStr">
-        <is>
-          <t>US region should be pre-selected by default</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="5" t="inlineStr">
-        <is>
-          <t>USR_032</t>
-        </is>
-      </c>
-      <c r="B34" s="5" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>Credentials - Select EU Region</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>Credentials screen displayed</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="inlineStr">
-        <is>
-          <t>Verify user can select EU region</t>
-        </is>
-      </c>
-      <c r="F34" s="5" t="inlineStr">
-        <is>
-          <t>1. Click on EU region option
-2. Observe selection state</t>
-        </is>
-      </c>
-      <c r="G34" s="5" t="inlineStr">
-        <is>
-          <t>EU region should be highlighted as selected, US deselected</t>
-        </is>
-      </c>
-      <c r="H34" s="5" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="5" t="inlineStr">
-        <is>
-          <t>USR_033</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>Credentials - Select IN Region</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>Credentials screen displayed</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>Verify user can select IN region</t>
-        </is>
-      </c>
-      <c r="F35" s="5" t="inlineStr">
-        <is>
-          <t>1. Click on IN region option
-2. Observe selection state</t>
-        </is>
-      </c>
-      <c r="G35" s="5" t="inlineStr">
-        <is>
-          <t>IN region should be highlighted as selected</t>
-        </is>
-      </c>
-      <c r="H35" s="5" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
-        <is>
-          <t>USR_034</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>Credentials - Enter Valid App ID</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>Credentials screen displayed</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
-        <is>
-          <t>Verify user can enter App ID</t>
-        </is>
-      </c>
-      <c r="F36" s="5" t="inlineStr">
-        <is>
-          <t>1. Click App ID input field
-2. Type valid App ID
-3. Observe input</t>
-        </is>
-      </c>
-      <c r="G36" s="5" t="inlineStr">
-        <is>
-          <t>App ID should be accepted and displayed in the field</t>
-        </is>
-      </c>
-      <c r="H36" s="5" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>USR_035</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>Credentials - Enter Valid Auth Key</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>Credentials screen displayed</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
-          <t>Verify user can enter Auth Key</t>
-        </is>
-      </c>
-      <c r="F37" s="5" t="inlineStr">
-        <is>
-          <t>1. Click Auth Key input field
-2. Type valid Auth Key
-3. Observe input</t>
-        </is>
-      </c>
-      <c r="G37" s="5" t="inlineStr">
-        <is>
-          <t>Auth Key should be accepted and displayed in the field</t>
-        </is>
-      </c>
-      <c r="H37" s="5" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
-        <is>
-          <t>USR_036</t>
-        </is>
-      </c>
-      <c r="B38" s="5" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>Credentials - Submit Valid Credentials</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>All fields filled with valid data</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="inlineStr">
-        <is>
-          <t>Verify successful submission navigates to login</t>
-        </is>
-      </c>
-      <c r="F38" s="5" t="inlineStr">
-        <is>
-          <t>1. Enter valid App ID
-2. Enter valid Auth Key
-3. Select region
-4. Click Continue</t>
-        </is>
-      </c>
-      <c r="G38" s="5" t="inlineStr">
-        <is>
-          <t>CometChat SDK should initialize and navigate to /login page</t>
-        </is>
-      </c>
-      <c r="H38" s="5" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr">
-        <is>
-          <t>USR_037</t>
-        </is>
-      </c>
-      <c r="B39" s="5" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>Credentials - LocalStorage Persistence</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>Valid credentials entered</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="inlineStr">
-        <is>
-          <t>Verify credentials are saved to localStorage</t>
-        </is>
-      </c>
-      <c r="F39" s="5" t="inlineStr">
-        <is>
-          <t>1. Enter App ID, Auth Key, select region
-2. Click Continue
-3. Check localStorage</t>
-        </is>
-      </c>
-      <c r="G39" s="5" t="inlineStr">
-        <is>
-          <t>region, appId, authKey should be stored in localStorage</t>
-        </is>
-      </c>
-      <c r="H39" s="5" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="5" t="inlineStr">
-        <is>
-          <t>USR_038</t>
-        </is>
-      </c>
-      <c r="B40" s="5" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>Credentials - Dark Mode Logo</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>Dark mode enabled on device</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
-          <t>Verify dark mode logo is displayed</t>
-        </is>
-      </c>
-      <c r="F40" s="5" t="inlineStr">
-        <is>
-          <t>1. Enable dark mode in OS settings
-2. Open credentials screen
-3. Observe logo</t>
-        </is>
-      </c>
-      <c r="G40" s="5" t="inlineStr">
-        <is>
-          <t>Dark mode CometChat logo should be displayed</t>
-        </is>
-      </c>
-      <c r="H40" s="5" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>USR_039</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>Credentials - Light Mode Logo</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>Light mode enabled on device</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>Verify light mode logo is displayed</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>1. Enable light mode in OS settings
-2. Open credentials screen
-3. Observe logo</t>
-        </is>
-      </c>
-      <c r="G41" s="2" t="inlineStr">
-        <is>
-          <t>Light mode CometChat logo should be displayed</t>
-        </is>
-      </c>
-      <c r="H41" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>USR_040</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>Login - Sample Users Display</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>Login screen loaded, API accessible</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>Verify sample users are fetched and displayed</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>1. Navigate to login screen
-2. Wait for users to load
-3. Observe user list</t>
-        </is>
-      </c>
-      <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t>Sample users should be fetched from API and displayed with avatar, name, and UID</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>USR_041</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>Login - Sample User Click Login</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>Sample users displayed</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t>Verify clicking a sample user logs in</t>
-        </is>
-      </c>
-      <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>1. Click on a sample user card
-2. Wait for login
-3. Observe navigation</t>
-        </is>
-      </c>
-      <c r="G43" s="2" t="inlineStr">
-        <is>
-          <t>User should be logged in via CometChatUIKit.login() and navigated to /home</t>
-        </is>
-      </c>
-      <c r="H43" s="2" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>USR_042</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>Login - Selection Indicator</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>Sample users displayed</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>Verify selected user shows selection indicator</t>
-        </is>
-      </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>1. Click on a sample user
-2. Observe visual feedback</t>
-        </is>
-      </c>
-      <c r="G44" s="2" t="inlineStr">
-        <is>
-          <t>Selected user should show a checked selection indicator circle</t>
-        </is>
-      </c>
-      <c r="H44" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>USR_043</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>Login - Custom UID Login</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>Login screen displayed</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>Verify login with custom UID</t>
-        </is>
-      </c>
-      <c r="F45" s="2" t="inlineStr">
-        <is>
-          <t>1. Enter a valid UID in the custom UID input
-2. Click Login button
-3. Wait for login</t>
-        </is>
-      </c>
-      <c r="G45" s="2" t="inlineStr">
-        <is>
-          <t>User should be logged in with the custom UID and navigated to /home</t>
-        </is>
-      </c>
-      <c r="H45" s="2" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>USR_044</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>Login - Change App Credentials Link</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>Login screen displayed</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>Verify Change App Credentials navigates to credentials screen</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>1. Click 'App Credentials' link text
-2. Observe navigation</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="inlineStr">
-        <is>
-          <t>Should clear localStorage credentials and navigate to /credentials</t>
-        </is>
-      </c>
-      <c r="H46" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>USR_045</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>Login - Auto-redirect If Logged In</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>User already logged in</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>Verify auto-redirect to home if already logged in</t>
-        </is>
-      </c>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
-          <t>1. Login successfully
-2. Navigate back to /login
-3. Observe behavior</t>
-        </is>
-      </c>
-      <c r="G47" s="2" t="inlineStr">
-        <is>
-          <t>Should automatically redirect to /home with replace:true</t>
-        </is>
-      </c>
-      <c r="H47" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>USR_046</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>Login - Fallback Sample Users</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>API endpoint unreachable</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>Verify fallback sample users are used when API fails</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>1. Block network to sample data API
-2. Navigate to login screen
-3. Observe user list</t>
-        </is>
-      </c>
-      <c r="G48" s="2" t="inlineStr">
-        <is>
-          <t>Fallback sample users from local sampledata.ts should be displayed</t>
-        </is>
-      </c>
-      <c r="H48" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>USR_047</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C49" s="2" t="inlineStr">
-        <is>
-          <t>Login - Dark Mode Logo</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>Dark mode enabled</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr">
-        <is>
-          <t>Verify dark mode logo on login screen</t>
-        </is>
-      </c>
-      <c r="F49" s="2" t="inlineStr">
-        <is>
-          <t>1. Enable dark mode
-2. Open login screen</t>
-        </is>
-      </c>
-      <c r="G49" s="2" t="inlineStr">
-        <is>
-          <t>Dark mode CometChat logo should be displayed</t>
-        </is>
-      </c>
-      <c r="H49" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>USR_048</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>User Details - Open Panel</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>User conversation selected</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>Verify user details panel opens on header click</t>
-        </is>
-      </c>
-      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>1. Select a user conversation
 2. Click on message header
 3. Observe side panel</t>
         </is>
       </c>
-      <c r="G50" s="2" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>User details side panel should open showing avatar, name, status</t>
         </is>
       </c>
-      <c r="H50" s="2" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>USR_049</t>
         </is>
       </c>
-      <c r="B51" s="2" t="inlineStr">
+      <c r="B34" s="5" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="C51" s="2" t="inlineStr">
+      <c r="C34" s="5" t="inlineStr">
         <is>
           <t>User Details - Block User Flow</t>
         </is>
       </c>
-      <c r="D51" s="2" t="inlineStr">
+      <c r="D34" s="5" t="inlineStr">
         <is>
           <t>User details panel open</t>
         </is>
       </c>
-      <c r="E51" s="2" t="inlineStr">
+      <c r="E34" s="5" t="inlineStr">
         <is>
           <t>Verify block user with confirmation dialog</t>
         </is>
       </c>
-      <c r="F51" s="2" t="inlineStr">
+      <c r="F34" s="5" t="inlineStr">
         <is>
           <t>1. Click Block option
 2. Observe confirmation dialog
 3. Click Block in dialog</t>
         </is>
       </c>
-      <c r="G51" s="2" t="inlineStr">
+      <c r="G34" s="5" t="inlineStr">
         <is>
           <t>Confirmation dialog appears, user blocked on confirm, toast shows 'Blocked successfully'</t>
         </is>
       </c>
-      <c r="H51" s="2" t="inlineStr">
+      <c r="H34" s="5" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>USR_050</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
+      <c r="B35" s="5" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr">
+      <c r="C35" s="5" t="inlineStr">
         <is>
           <t>User Details - Unblock User</t>
         </is>
       </c>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="D35" s="5" t="inlineStr">
         <is>
           <t>User is blocked, details panel open</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="E35" s="5" t="inlineStr">
         <is>
           <t>Verify unblock user action</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr">
+      <c r="F35" s="5" t="inlineStr">
         <is>
           <t>1. Click Unblock option in details
 2. Observe behavior</t>
         </is>
       </c>
-      <c r="G52" s="2" t="inlineStr">
+      <c r="G35" s="5" t="inlineStr">
         <is>
           <t>User should be unblocked immediately (no confirmation), action text changes to Block</t>
         </is>
       </c>
-      <c r="H52" s="2" t="inlineStr">
+      <c r="H35" s="5" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>USR_051</t>
         </is>
       </c>
-      <c r="B53" s="2" t="inlineStr">
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="C53" s="2" t="inlineStr">
+      <c r="C36" s="5" t="inlineStr">
         <is>
           <t>User Details - Block Hides Status</t>
         </is>
       </c>
-      <c r="D53" s="2" t="inlineStr">
+      <c r="D36" s="5" t="inlineStr">
         <is>
           <t>User details panel open</t>
         </is>
       </c>
-      <c r="E53" s="2" t="inlineStr">
+      <c r="E36" s="5" t="inlineStr">
         <is>
           <t>Verify blocking hides user status</t>
         </is>
       </c>
-      <c r="F53" s="2" t="inlineStr">
+      <c r="F36" s="5" t="inlineStr">
         <is>
           <t>1. Block a user
 2. Observe status indicator</t>
         </is>
       </c>
-      <c r="G53" s="2" t="inlineStr">
+      <c r="G36" s="5" t="inlineStr">
         <is>
           <t>User status (online/offline) should be hidden after blocking</t>
         </is>
       </c>
-      <c r="H53" s="2" t="inlineStr">
+      <c r="H36" s="5" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>USR_052</t>
         </is>
       </c>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="B37" s="5" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr">
+      <c r="C37" s="5" t="inlineStr">
         <is>
           <t>User Details - Unblock Shows Status</t>
         </is>
       </c>
-      <c r="D54" s="2" t="inlineStr">
+      <c r="D37" s="5" t="inlineStr">
         <is>
           <t>Blocked user details panel open</t>
         </is>
       </c>
-      <c r="E54" s="2" t="inlineStr">
+      <c r="E37" s="5" t="inlineStr">
         <is>
           <t>Verify unblocking restores status visibility</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
+      <c r="F37" s="5" t="inlineStr">
         <is>
           <t>1. Unblock a user
 2. Observe status indicator</t>
         </is>
       </c>
-      <c r="G54" s="2" t="inlineStr">
+      <c r="G37" s="5" t="inlineStr">
         <is>
           <t>User status should become visible again after unblocking</t>
         </is>
       </c>
-      <c r="H54" s="2" t="inlineStr">
+      <c r="H37" s="5" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>USR_053</t>
         </is>
       </c>
-      <c r="B55" s="2" t="inlineStr">
+      <c r="B38" s="5" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr">
+      <c r="C38" s="5" t="inlineStr">
         <is>
           <t>User Details - Delete Chat</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
+      <c r="D38" s="5" t="inlineStr">
         <is>
           <t>User details panel open, conversation exists</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr">
+      <c r="E38" s="5" t="inlineStr">
         <is>
           <t>Verify delete chat with confirmation</t>
         </is>
       </c>
-      <c r="F55" s="2" t="inlineStr">
+      <c r="F38" s="5" t="inlineStr">
         <is>
           <t>1. Click Delete Chat
 2. Observe confirmation dialog
 3. Confirm deletion</t>
         </is>
       </c>
-      <c r="G55" s="2" t="inlineStr">
+      <c r="G38" s="5" t="inlineStr">
         <is>
           <t>Confirmation dialog appears, conversation deleted, side panel closes, toast shown</t>
         </is>
       </c>
-      <c r="H55" s="2" t="inlineStr">
+      <c r="H38" s="5" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="2" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t>USR_054</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr">
+      <c r="B39" s="5" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr">
+      <c r="C39" s="5" t="inlineStr">
         <is>
           <t>User Details - Close Panel</t>
         </is>
       </c>
-      <c r="D56" s="2" t="inlineStr">
+      <c r="D39" s="5" t="inlineStr">
         <is>
           <t>User details panel open</t>
         </is>
       </c>
-      <c r="E56" s="2" t="inlineStr">
+      <c r="E39" s="5" t="inlineStr">
         <is>
           <t>Verify closing the details panel</t>
         </is>
       </c>
-      <c r="F56" s="2" t="inlineStr">
+      <c r="F39" s="5" t="inlineStr">
         <is>
           <t>1. Click close icon on panel
 2. Observe behavior</t>
         </is>
       </c>
-      <c r="G56" s="2" t="inlineStr">
+      <c r="G39" s="5" t="inlineStr">
         <is>
           <t>Side panel should close, messages view remains</t>
         </is>
       </c>
-      <c r="H56" s="2" t="inlineStr">
+      <c r="H39" s="5" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="2" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>USR_055</t>
         </is>
       </c>
-      <c r="B57" s="2" t="inlineStr">
+      <c r="B40" s="5" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="C57" s="2" t="inlineStr">
+      <c r="C40" s="5" t="inlineStr">
         <is>
           <t>User Details - Block Confirmation Cancel</t>
         </is>
       </c>
-      <c r="D57" s="2" t="inlineStr">
+      <c r="D40" s="5" t="inlineStr">
         <is>
           <t>Block confirmation dialog shown</t>
         </is>
       </c>
-      <c r="E57" s="2" t="inlineStr">
+      <c r="E40" s="5" t="inlineStr">
         <is>
           <t>Verify canceling block confirmation</t>
         </is>
       </c>
-      <c r="F57" s="2" t="inlineStr">
+      <c r="F40" s="5" t="inlineStr">
         <is>
           <t>1. Click Block
 2. In confirmation dialog click Cancel</t>
         </is>
       </c>
-      <c r="G57" s="2" t="inlineStr">
+      <c r="G40" s="5" t="inlineStr">
         <is>
           <t>Dialog should close, user remains unblocked</t>
         </is>
       </c>
-      <c r="H57" s="2" t="inlineStr">
+      <c r="H40" s="5" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>USR_056</t>
         </is>
       </c>
-      <c r="B58" s="2" t="inlineStr">
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>User Details - Delete Chat Confirmation Cancel</t>
         </is>
       </c>
-      <c r="D58" s="2" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>Delete confirmation dialog shown</t>
         </is>
       </c>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="E41" s="2" t="inlineStr">
         <is>
           <t>Verify canceling delete confirmation</t>
         </is>
       </c>
-      <c r="F58" s="2" t="inlineStr">
+      <c r="F41" s="2" t="inlineStr">
         <is>
           <t>1. Click Delete Chat
 2. In confirmation dialog click Cancel</t>
         </is>
       </c>
-      <c r="G58" s="2" t="inlineStr">
+      <c r="G41" s="2" t="inlineStr">
         <is>
           <t>Dialog should close, conversation remains</t>
         </is>
       </c>
-      <c r="H58" s="2" t="inlineStr">
+      <c r="H41" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="2" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="8" t="n"/>
+      <c r="B42" s="8" t="n"/>
+      <c r="C42" s="8" t="n"/>
+      <c r="D42" s="8" t="n"/>
+      <c r="E42" s="8" t="n"/>
+      <c r="F42" s="8" t="n"/>
+      <c r="G42" s="8" t="n"/>
+      <c r="H42" s="8" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>USERS_005</t>
         </is>
       </c>
-      <c r="B60" s="2" t="inlineStr">
+      <c r="B43" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="C60" s="2" t="inlineStr">
+      <c r="C43" s="2" t="inlineStr">
         <is>
           <t>Verify Users List display</t>
         </is>
       </c>
-      <c r="D60" s="2" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>User is logged in, no users exist</t>
         </is>
       </c>
-      <c r="E60" s="2" t="inlineStr">
+      <c r="E43" s="2" t="inlineStr">
         <is>
           <t>Verify empty users list state</t>
         </is>
       </c>
-      <c r="F60" s="2" t="inlineStr">
+      <c r="F43" s="2" t="inlineStr">
         <is>
           <t>1. Navigate to Users tab with no users in system.
 2. Observe display.</t>
         </is>
       </c>
-      <c r="G60" s="2" t="inlineStr">
+      <c r="G43" s="2" t="inlineStr">
         <is>
           <t>Appropriate empty state message should display (e.g., "No users found").</t>
         </is>
       </c>
-      <c r="H60" s="2" t="inlineStr">
+      <c r="H43" s="2" t="inlineStr">
         <is>
           <t>Medium / Medium</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="2" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>USERS_014</t>
         </is>
       </c>
-      <c r="B61" s="2" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="C61" s="2" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t>Verify Search functionality</t>
         </is>
       </c>
-      <c r="D61" s="2" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>User is logged in and on Users tab</t>
         </is>
       </c>
-      <c r="E61" s="2" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>Verify search with no matching results</t>
         </is>
       </c>
-      <c r="F61" s="2" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>1. Navigate to Users tab.
 2. Type "XYZ123" in search field.
 3. Observe results.</t>
         </is>
       </c>
-      <c r="G61" s="2" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>Empty state should display with message like "No users found" or "No results".</t>
         </is>
       </c>
-      <c r="H61" s="2" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr">
         <is>
           <t>Medium / Medium</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="2" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>USERS_024</t>
         </is>
       </c>
-      <c r="B62" s="2" t="inlineStr">
+      <c r="B45" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="C62" s="2" t="inlineStr">
+      <c r="C45" s="2" t="inlineStr">
         <is>
           <t>Verify Users List loading</t>
         </is>
       </c>
-      <c r="D62" s="2" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>User is logged in, slow network</t>
         </is>
       </c>
-      <c r="E62" s="2" t="inlineStr">
+      <c r="E45" s="2" t="inlineStr">
         <is>
           <t>Verify loading state during slow connection</t>
         </is>
       </c>
-      <c r="F62" s="2" t="inlineStr">
+      <c r="F45" s="2" t="inlineStr">
         <is>
           <t>1. Simulate slow network.
 2. Navigate to Users tab.
 3. Observe loading behavior.</t>
         </is>
       </c>
-      <c r="G62" s="2" t="inlineStr">
+      <c r="G45" s="2" t="inlineStr">
         <is>
           <t>Loading indicator should display while users list is being fetched.</t>
         </is>
       </c>
-      <c r="H62" s="2" t="inlineStr">
+      <c r="H45" s="2" t="inlineStr">
         <is>
           <t>Medium / Medium</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="2" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>USR_010</t>
         </is>
       </c>
-      <c r="B63" s="2" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="C63" s="2" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>Block - Already Blocked</t>
         </is>
       </c>
-      <c r="D63" s="2" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>User already blocked</t>
         </is>
       </c>
-      <c r="E63" s="2" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>Verify block option changes to unblock</t>
         </is>
       </c>
-      <c r="F63" s="2" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>1. Check blocked user options</t>
         </is>
       </c>
-      <c r="G63" s="2" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>Only unblock option shown, not block</t>
         </is>
       </c>
-      <c r="H63" s="2" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
         <is>
           <t>USR_011</t>
         </is>
       </c>
-      <c r="B64" s="2" t="inlineStr">
+      <c r="B47" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="C64" s="2" t="inlineStr">
+      <c r="C47" s="2" t="inlineStr">
         <is>
           <t>View Profile - No Profile</t>
         </is>
       </c>
-      <c r="D64" s="2" t="inlineStr">
+      <c r="D47" s="2" t="inlineStr">
         <is>
           <t>User has minimal profile</t>
         </is>
       </c>
-      <c r="E64" s="2" t="inlineStr">
+      <c r="E47" s="2" t="inlineStr">
         <is>
           <t>Verify handling of empty profile data</t>
         </is>
       </c>
-      <c r="F64" s="2" t="inlineStr">
+      <c r="F47" s="2" t="inlineStr">
         <is>
           <t>1. View profile of user with no details</t>
         </is>
       </c>
-      <c r="G64" s="2" t="inlineStr">
+      <c r="G47" s="2" t="inlineStr">
         <is>
           <t>Appropriate fallback/empty state shown</t>
         </is>
       </c>
-      <c r="H64" s="2" t="inlineStr">
+      <c r="H47" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="2" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>USR_012</t>
         </is>
       </c>
-      <c r="B65" s="2" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="C65" s="2" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>User Status Hidden</t>
         </is>
       </c>
-      <c r="D65" s="2" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>hideUserStatus=true</t>
         </is>
       </c>
-      <c r="E65" s="2" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>Verify status indicator hidden</t>
         </is>
       </c>
-      <c r="F65" s="2" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>1. Set hideUserStatus=true
 2. Check users</t>
         </is>
       </c>
-      <c r="G65" s="2" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
         <is>
           <t>No online/offline indicators visible</t>
         </is>
       </c>
-      <c r="H65" s="2" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="2" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>USR_013</t>
         </is>
       </c>
-      <c r="B66" s="2" t="inlineStr">
+      <c r="B49" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
         <is>
           <t>Block Self</t>
         </is>
       </c>
-      <c r="D66" s="2" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>Own profile</t>
         </is>
       </c>
-      <c r="E66" s="2" t="inlineStr">
+      <c r="E49" s="2" t="inlineStr">
         <is>
           <t>Verify cannot block self</t>
         </is>
       </c>
-      <c r="F66" s="2" t="inlineStr">
+      <c r="F49" s="2" t="inlineStr">
         <is>
           <t>1. Check own profile options</t>
         </is>
       </c>
-      <c r="G66" s="2" t="inlineStr">
+      <c r="G49" s="2" t="inlineStr">
         <is>
           <t>Block option not available for self</t>
         </is>
       </c>
-      <c r="H66" s="2" t="inlineStr">
+      <c r="H49" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="2" t="inlineStr">
-        <is>
-          <t>USR_057</t>
-        </is>
-      </c>
-      <c r="B67" s="2" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>USR_064</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="C67" s="2" t="inlineStr">
-        <is>
-          <t>Credentials - Empty App ID</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="inlineStr">
-        <is>
-          <t>Credentials screen displayed</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="inlineStr">
-        <is>
-          <t>Verify form validation for empty App ID</t>
-        </is>
-      </c>
-      <c r="F67" s="2" t="inlineStr">
-        <is>
-          <t>1. Leave App ID empty
-2. Enter Auth Key
-3. Click Continue</t>
-        </is>
-      </c>
-      <c r="G67" s="2" t="inlineStr">
-        <is>
-          <t>Form should not submit, HTML5 required validation should trigger</t>
-        </is>
-      </c>
-      <c r="H67" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="2" t="inlineStr">
-        <is>
-          <t>USR_058</t>
-        </is>
-      </c>
-      <c r="B68" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>Credentials - Empty Auth Key</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="inlineStr">
-        <is>
-          <t>Credentials screen displayed</t>
-        </is>
-      </c>
-      <c r="E68" s="2" t="inlineStr">
-        <is>
-          <t>Verify form validation for empty Auth Key</t>
-        </is>
-      </c>
-      <c r="F68" s="2" t="inlineStr">
-        <is>
-          <t>1. Enter App ID
-2. Leave Auth Key empty
-3. Click Continue</t>
-        </is>
-      </c>
-      <c r="G68" s="2" t="inlineStr">
-        <is>
-          <t>Form should not submit, HTML5 required validation should trigger</t>
-        </is>
-      </c>
-      <c r="H68" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="2" t="inlineStr">
-        <is>
-          <t>USR_059</t>
-        </is>
-      </c>
-      <c r="B69" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="C69" s="2" t="inlineStr">
-        <is>
-          <t>Credentials - Invalid App ID</t>
-        </is>
-      </c>
-      <c r="D69" s="2" t="inlineStr">
-        <is>
-          <t>Credentials screen displayed</t>
-        </is>
-      </c>
-      <c r="E69" s="2" t="inlineStr">
-        <is>
-          <t>Verify error handling for invalid App ID</t>
-        </is>
-      </c>
-      <c r="F69" s="2" t="inlineStr">
-        <is>
-          <t>1. Enter invalid/random App ID
-2. Enter valid Auth Key
-3. Click Continue</t>
-        </is>
-      </c>
-      <c r="G69" s="2" t="inlineStr">
-        <is>
-          <t>SDK initialization should fail, appropriate error handling</t>
-        </is>
-      </c>
-      <c r="H69" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="2" t="inlineStr">
-        <is>
-          <t>USR_060</t>
-        </is>
-      </c>
-      <c r="B70" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="C70" s="2" t="inlineStr">
-        <is>
-          <t>Credentials - Both Fields Empty</t>
-        </is>
-      </c>
-      <c r="D70" s="2" t="inlineStr">
-        <is>
-          <t>Credentials screen displayed</t>
-        </is>
-      </c>
-      <c r="E70" s="2" t="inlineStr">
-        <is>
-          <t>Verify form won't submit with all fields empty</t>
-        </is>
-      </c>
-      <c r="F70" s="2" t="inlineStr">
-        <is>
-          <t>1. Leave all fields empty
-2. Click Continue</t>
-        </is>
-      </c>
-      <c r="G70" s="2" t="inlineStr">
-        <is>
-          <t>Form should not submit due to required field validation</t>
-        </is>
-      </c>
-      <c r="H70" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="2" t="inlineStr">
-        <is>
-          <t>USR_061</t>
-        </is>
-      </c>
-      <c r="B71" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="C71" s="2" t="inlineStr">
-        <is>
-          <t>Login - Empty Custom UID</t>
-        </is>
-      </c>
-      <c r="D71" s="2" t="inlineStr">
-        <is>
-          <t>Login screen displayed</t>
-        </is>
-      </c>
-      <c r="E71" s="2" t="inlineStr">
-        <is>
-          <t>Verify empty UID validation</t>
-        </is>
-      </c>
-      <c r="F71" s="2" t="inlineStr">
-        <is>
-          <t>1. Leave UID field empty
-2. Click Login</t>
-        </is>
-      </c>
-      <c r="G71" s="2" t="inlineStr">
-        <is>
-          <t>Form should not submit due to required field validation</t>
-        </is>
-      </c>
-      <c r="H71" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="2" t="inlineStr">
-        <is>
-          <t>USR_062</t>
-        </is>
-      </c>
-      <c r="B72" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="C72" s="2" t="inlineStr">
-        <is>
-          <t>Login - Invalid Custom UID</t>
-        </is>
-      </c>
-      <c r="D72" s="2" t="inlineStr">
-        <is>
-          <t>Login screen displayed</t>
-        </is>
-      </c>
-      <c r="E72" s="2" t="inlineStr">
-        <is>
-          <t>Verify login with non-existent UID</t>
-        </is>
-      </c>
-      <c r="F72" s="2" t="inlineStr">
-        <is>
-          <t>1. Enter non-existent UID
-2. Click Login</t>
-        </is>
-      </c>
-      <c r="G72" s="2" t="inlineStr">
-        <is>
-          <t>Login should fail, error logged to console</t>
-        </is>
-      </c>
-      <c r="H72" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="2" t="inlineStr">
-        <is>
-          <t>USR_063</t>
-        </is>
-      </c>
-      <c r="B73" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="C73" s="2" t="inlineStr">
-        <is>
-          <t>Login - No Credentials Redirect</t>
-        </is>
-      </c>
-      <c r="D73" s="2" t="inlineStr">
-        <is>
-          <t>No credentials in localStorage or AppConstants</t>
-        </is>
-      </c>
-      <c r="E73" s="2" t="inlineStr">
-        <is>
-          <t>Verify redirect to credentials when no credentials exist</t>
-        </is>
-      </c>
-      <c r="F73" s="2" t="inlineStr">
-        <is>
-          <t>1. Clear all localStorage
-2. Set empty AppConstants
-3. Navigate to /login</t>
-        </is>
-      </c>
-      <c r="G73" s="2" t="inlineStr">
-        <is>
-          <t>Should redirect to /credentials screen</t>
-        </is>
-      </c>
-      <c r="H73" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="2" t="inlineStr">
-        <is>
-          <t>USR_064</t>
-        </is>
-      </c>
-      <c r="B74" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="C74" s="2" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr">
         <is>
           <t>User Details - Delete Fresh Chat</t>
         </is>
       </c>
-      <c r="D74" s="2" t="inlineStr">
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>Fresh chat with no messages</t>
         </is>
       </c>
-      <c r="E74" s="2" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>Verify delete chat disabled for fresh chats</t>
         </is>
       </c>
-      <c r="F74" s="2" t="inlineStr">
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>1. Start new chat (no messages sent)
 2. Open details
 3. Observe Delete Chat</t>
         </is>
       </c>
-      <c r="G74" s="2" t="inlineStr">
+      <c r="G50" s="2" t="inlineStr">
         <is>
           <t>Delete Chat option should be visually disabled (action-item-disabled class)</t>
         </is>
       </c>
-      <c r="H74" s="2" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="2" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
         <is>
           <t>USR_065</t>
         </is>
       </c>
-      <c r="B75" s="2" t="inlineStr">
+      <c r="B51" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="C75" s="2" t="inlineStr">
+      <c r="C51" s="2" t="inlineStr">
         <is>
           <t>User Details - Delete Chat API Failure</t>
         </is>
       </c>
-      <c r="D75" s="2" t="inlineStr">
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>User details panel open</t>
         </is>
       </c>
-      <c r="E75" s="2" t="inlineStr">
+      <c r="E51" s="2" t="inlineStr">
         <is>
           <t>Verify error handling on delete chat failure</t>
         </is>
       </c>
-      <c r="F75" s="2" t="inlineStr">
+      <c r="F51" s="2" t="inlineStr">
         <is>
           <t>1. Click Delete Chat
 2. Confirm
 3. Simulate API failure</t>
         </is>
       </c>
-      <c r="G75" s="2" t="inlineStr">
+      <c r="G51" s="2" t="inlineStr">
         <is>
           <t>Error should be caught and logged, app should not crash</t>
         </is>
       </c>
-      <c r="H75" s="2" t="inlineStr">
+      <c r="H51" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="n"/>
+      <c r="B52" s="8" t="n"/>
+      <c r="C52" s="8" t="n"/>
+      <c r="D52" s="8" t="n"/>
+      <c r="E52" s="8" t="n"/>
+      <c r="F52" s="8" t="n"/>
+      <c r="G52" s="8" t="n"/>
+      <c r="H52" s="8" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="n"/>
+      <c r="B53" s="8" t="n"/>
+      <c r="C53" s="8" t="n"/>
+      <c r="D53" s="8" t="n"/>
+      <c r="E53" s="8" t="n"/>
+      <c r="F53" s="8" t="n"/>
+      <c r="G53" s="8" t="n"/>
+      <c r="H53" s="8" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="n"/>
+      <c r="B54" s="8" t="n"/>
+      <c r="C54" s="8" t="n"/>
+      <c r="D54" s="8" t="n"/>
+      <c r="E54" s="8" t="n"/>
+      <c r="F54" s="8" t="n"/>
+      <c r="G54" s="8" t="n"/>
+      <c r="H54" s="8" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="n"/>
+      <c r="B55" s="8" t="n"/>
+      <c r="C55" s="8" t="n"/>
+      <c r="D55" s="8" t="n"/>
+      <c r="E55" s="8" t="n"/>
+      <c r="F55" s="8" t="n"/>
+      <c r="G55" s="8" t="n"/>
+      <c r="H55" s="8" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="n"/>
+      <c r="B56" s="8" t="n"/>
+      <c r="C56" s="8" t="n"/>
+      <c r="D56" s="8" t="n"/>
+      <c r="E56" s="8" t="n"/>
+      <c r="F56" s="8" t="n"/>
+      <c r="G56" s="8" t="n"/>
+      <c r="H56" s="8" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="n"/>
+      <c r="B57" s="8" t="n"/>
+      <c r="C57" s="8" t="n"/>
+      <c r="D57" s="8" t="n"/>
+      <c r="E57" s="8" t="n"/>
+      <c r="F57" s="8" t="n"/>
+      <c r="G57" s="8" t="n"/>
+      <c r="H57" s="8" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="n"/>
+      <c r="B58" s="8" t="n"/>
+      <c r="C58" s="8" t="n"/>
+      <c r="D58" s="8" t="n"/>
+      <c r="E58" s="8" t="n"/>
+      <c r="F58" s="8" t="n"/>
+      <c r="G58" s="8" t="n"/>
+      <c r="H58" s="8" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="7" t="n"/>
+      <c r="B59" s="7" t="n"/>
+      <c r="C59" s="7" t="n"/>
+      <c r="D59" s="7" t="n"/>
+      <c r="E59" s="7" t="n"/>
+      <c r="F59" s="7" t="n"/>
+      <c r="G59" s="7" t="n"/>
+      <c r="H59" s="7" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="n"/>
+      <c r="B60" s="8" t="n"/>
+      <c r="C60" s="8" t="n"/>
+      <c r="D60" s="8" t="n"/>
+      <c r="E60" s="8" t="n"/>
+      <c r="F60" s="8" t="n"/>
+      <c r="G60" s="8" t="n"/>
+      <c r="H60" s="8" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="8" t="n"/>
+      <c r="B61" s="8" t="n"/>
+      <c r="C61" s="8" t="n"/>
+      <c r="D61" s="8" t="n"/>
+      <c r="E61" s="8" t="n"/>
+      <c r="F61" s="8" t="n"/>
+      <c r="G61" s="8" t="n"/>
+      <c r="H61" s="8" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="8" t="n"/>
+      <c r="B62" s="8" t="n"/>
+      <c r="C62" s="8" t="n"/>
+      <c r="D62" s="8" t="n"/>
+      <c r="E62" s="8" t="n"/>
+      <c r="F62" s="8" t="n"/>
+      <c r="G62" s="8" t="n"/>
+      <c r="H62" s="8" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="8" t="n"/>
+      <c r="B63" s="8" t="n"/>
+      <c r="C63" s="8" t="n"/>
+      <c r="D63" s="8" t="n"/>
+      <c r="E63" s="8" t="n"/>
+      <c r="F63" s="8" t="n"/>
+      <c r="G63" s="8" t="n"/>
+      <c r="H63" s="8" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="8" t="n"/>
+      <c r="B64" s="8" t="n"/>
+      <c r="C64" s="8" t="n"/>
+      <c r="D64" s="8" t="n"/>
+      <c r="E64" s="8" t="n"/>
+      <c r="F64" s="8" t="n"/>
+      <c r="G64" s="8" t="n"/>
+      <c r="H64" s="8" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="8" t="n"/>
+      <c r="B65" s="8" t="n"/>
+      <c r="C65" s="8" t="n"/>
+      <c r="D65" s="8" t="n"/>
+      <c r="E65" s="8" t="n"/>
+      <c r="F65" s="8" t="n"/>
+      <c r="G65" s="8" t="n"/>
+      <c r="H65" s="8" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="8" t="n"/>
+      <c r="B66" s="8" t="n"/>
+      <c r="C66" s="8" t="n"/>
+      <c r="D66" s="8" t="n"/>
+      <c r="E66" s="8" t="n"/>
+      <c r="F66" s="8" t="n"/>
+      <c r="G66" s="8" t="n"/>
+      <c r="H66" s="8" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="8" t="n"/>
+      <c r="B67" s="8" t="n"/>
+      <c r="C67" s="8" t="n"/>
+      <c r="D67" s="8" t="n"/>
+      <c r="E67" s="8" t="n"/>
+      <c r="F67" s="8" t="n"/>
+      <c r="G67" s="8" t="n"/>
+      <c r="H67" s="8" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="8" t="n"/>
+      <c r="B68" s="8" t="n"/>
+      <c r="C68" s="8" t="n"/>
+      <c r="D68" s="8" t="n"/>
+      <c r="E68" s="8" t="n"/>
+      <c r="F68" s="8" t="n"/>
+      <c r="G68" s="8" t="n"/>
+      <c r="H68" s="8" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="8" t="n"/>
+      <c r="B69" s="8" t="n"/>
+      <c r="C69" s="8" t="n"/>
+      <c r="D69" s="8" t="n"/>
+      <c r="E69" s="8" t="n"/>
+      <c r="F69" s="8" t="n"/>
+      <c r="G69" s="8" t="n"/>
+      <c r="H69" s="8" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="8" t="n"/>
+      <c r="B70" s="8" t="n"/>
+      <c r="C70" s="8" t="n"/>
+      <c r="D70" s="8" t="n"/>
+      <c r="E70" s="8" t="n"/>
+      <c r="F70" s="8" t="n"/>
+      <c r="G70" s="8" t="n"/>
+      <c r="H70" s="8" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="8" t="n"/>
+      <c r="B71" s="8" t="n"/>
+      <c r="C71" s="8" t="n"/>
+      <c r="D71" s="8" t="n"/>
+      <c r="E71" s="8" t="n"/>
+      <c r="F71" s="8" t="n"/>
+      <c r="G71" s="8" t="n"/>
+      <c r="H71" s="8" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="8" t="n"/>
+      <c r="B72" s="8" t="n"/>
+      <c r="C72" s="8" t="n"/>
+      <c r="D72" s="8" t="n"/>
+      <c r="E72" s="8" t="n"/>
+      <c r="F72" s="8" t="n"/>
+      <c r="G72" s="8" t="n"/>
+      <c r="H72" s="8" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="8" t="n"/>
+      <c r="B73" s="8" t="n"/>
+      <c r="C73" s="8" t="n"/>
+      <c r="D73" s="8" t="n"/>
+      <c r="E73" s="8" t="n"/>
+      <c r="F73" s="8" t="n"/>
+      <c r="G73" s="8" t="n"/>
+      <c r="H73" s="8" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="8" t="n"/>
+      <c r="B74" s="8" t="n"/>
+      <c r="C74" s="8" t="n"/>
+      <c r="D74" s="8" t="n"/>
+      <c r="E74" s="8" t="n"/>
+      <c r="F74" s="8" t="n"/>
+      <c r="G74" s="8" t="n"/>
+      <c r="H74" s="8" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="8" t="n"/>
+      <c r="B75" s="8" t="n"/>
+      <c r="C75" s="8" t="n"/>
+      <c r="D75" s="8" t="n"/>
+      <c r="E75" s="8" t="n"/>
+      <c r="F75" s="8" t="n"/>
+      <c r="G75" s="8" t="n"/>
+      <c r="H75" s="8" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="7" t="n"/>
+      <c r="B76" s="7" t="n"/>
+      <c r="C76" s="7" t="n"/>
+      <c r="D76" s="7" t="n"/>
+      <c r="E76" s="7" t="n"/>
+      <c r="F76" s="7" t="n"/>
+      <c r="G76" s="7" t="n"/>
+      <c r="H76" s="7" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3541,7 +2758,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3805,7 +3022,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>USR_066</t>
+          <t>USR_070</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -3815,29 +3032,28 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Credentials - SDK Init Integration</t>
+          <t>User Details - Block Event Propagation</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Valid credentials available</t>
+          <t>User blocked from details</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Verify CometChat SDK initializes with provided credentials</t>
+          <t>Verify block event updates message composer</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>1. Enter valid App ID, Auth Key, region
-2. Click Continue
-3. Monitor SDK init</t>
+          <t>1. Block user from details panel
+2. Observe message composer</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>UIKitSettingsBuilder should build with correct params, SDK init succeeds</t>
+          <t>Composer should be replaced with 'Cannot send to blocked user' message with unblock link</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -3849,7 +3065,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>USR_067</t>
+          <t>USR_071</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -3859,40 +3075,40 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Credentials - Navigation to Login</t>
+          <t>User Details - Unblock Event Propagation</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>SDK initialized successfully</t>
+          <t>User unblocked from details</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Verify navigation from credentials to login screen</t>
+          <t>Verify unblock event restores composer</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>1. Submit valid credentials
-2. Observe navigation</t>
+          <t>1. Unblock user from details
+2. Observe message composer</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>App should navigate to /login route with replace:true</t>
+          <t>Message composer should reappear, blocked message removed</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>USR_068</t>
+          <t>USR_072</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -3902,40 +3118,40 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Login - CometChatUIKit.login Integration</t>
+          <t>User Details - Delete Conversation Event</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Valid UID available</t>
+          <t>Chat deleted from details</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Verify CometChatUIKit.login() is called correctly</t>
+          <t>Verify conversation deleted event fires</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>1. Click sample user or enter custom UID
-2. Monitor SDK login call</t>
+          <t>1. Delete chat from details
+2. Monitor events</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>CometChatUIKit.login(uid) should be called and return loggedInUser</t>
+          <t>ccConversationDeleted event should fire, conversation removed from list</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>USR_069</t>
+          <t>USR_073</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -3945,294 +3161,148 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Login - Sample Users API Integration</t>
+          <t>User Details - Block Toast Notification</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Network available</t>
+          <t>User blocked</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Verify sample users fetched from correct API endpoint</t>
+          <t>Verify toast notification on block</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>1. Open login screen
-2. Monitor network requests</t>
+          <t>1. Block a user
+2. Observe toast</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>GET request to https://assets.cc-cluster-2.io/sampleapp/v2/sampledata.json should be made</t>
+          <t>Toast should show 'Blocked successfully' message</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>USR_070</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>User Details - Block Event Propagation</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>User blocked from details</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Verify block event updates message composer</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>1. Block user from details panel
-2. Observe message composer</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Composer should be replaced with 'Cannot send to blocked user' message with unblock link</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
+      <c r="A11" s="8" t="n"/>
+      <c r="B11" s="8" t="n"/>
+      <c r="C11" s="8" t="n"/>
+      <c r="D11" s="8" t="n"/>
+      <c r="E11" s="8" t="n"/>
+      <c r="F11" s="8" t="n"/>
+      <c r="G11" s="8" t="n"/>
+      <c r="H11" s="8" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>USR_071</t>
+          <t>USR_017</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>User Details - Unblock Event Propagation</t>
+          <t>Block + Incoming Messages</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>User unblocked from details</t>
+          <t>User blocked</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Verify unblock event restores composer</t>
+          <t>Verify blocked user messages not received</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>1. Unblock user from details
-2. Observe message composer</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>Message composer should reappear, blocked message removed</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>USR_072</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>User Details - Delete Conversation Event</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Chat deleted from details</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Verify conversation deleted event fires</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>1. Delete chat from details
-2. Monitor events</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>ccConversationDeleted event should fire, conversation removed from list</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>USR_073</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>User Details - Block Toast Notification</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>User blocked</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Verify toast notification on block</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>1. Block a user
-2. Observe toast</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>Toast should show 'Blocked successfully' message</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>USR_017</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Block + Incoming Messages</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>User blocked</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Verify blocked user messages not received</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>1. Block user
 2. Blocked user sends message</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Message not received or shown</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="8" t="n"/>
+      <c r="B13" s="8" t="n"/>
+      <c r="C13" s="8" t="n"/>
+      <c r="D13" s="8" t="n"/>
+      <c r="E13" s="8" t="n"/>
+      <c r="F13" s="8" t="n"/>
+      <c r="G13" s="8" t="n"/>
+      <c r="H13" s="8" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="n"/>
+      <c r="B14" s="8" t="n"/>
+      <c r="C14" s="8" t="n"/>
+      <c r="D14" s="8" t="n"/>
+      <c r="E14" s="8" t="n"/>
+      <c r="F14" s="8" t="n"/>
+      <c r="G14" s="8" t="n"/>
+      <c r="H14" s="8" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="n"/>
+      <c r="B15" s="7" t="n"/>
+      <c r="C15" s="7" t="n"/>
+      <c r="D15" s="7" t="n"/>
+      <c r="E15" s="7" t="n"/>
+      <c r="F15" s="7" t="n"/>
+      <c r="G15" s="7" t="n"/>
+      <c r="H15" s="7" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="n"/>
+      <c r="B16" s="8" t="n"/>
+      <c r="C16" s="8" t="n"/>
+      <c r="D16" s="8" t="n"/>
+      <c r="E16" s="8" t="n"/>
+      <c r="F16" s="8" t="n"/>
+      <c r="G16" s="8" t="n"/>
+      <c r="H16" s="8" t="n"/>
+    </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>USR_074</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Credentials - SDK Init Failure</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Invalid credentials entered</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>Verify app handles SDK initialization failure</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>1. Enter invalid credentials
-2. Click Continue
-3. Observe behavior</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>App should handle error gracefully without crashing</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
+      <c r="A17" s="8" t="n"/>
+      <c r="B17" s="8" t="n"/>
+      <c r="C17" s="8" t="n"/>
+      <c r="D17" s="8" t="n"/>
+      <c r="E17" s="8" t="n"/>
+      <c r="F17" s="8" t="n"/>
+      <c r="G17" s="8" t="n"/>
+      <c r="H17" s="8" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="n"/>
+      <c r="B18" s="7" t="n"/>
+      <c r="C18" s="7" t="n"/>
+      <c r="D18" s="7" t="n"/>
+      <c r="E18" s="7" t="n"/>
+      <c r="F18" s="7" t="n"/>
+      <c r="G18" s="7" t="n"/>
+      <c r="H18" s="7" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4246,7 +3316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4527,7 +3597,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>USR_075</t>
+          <t>USR_077</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -4537,109 +3607,20 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Credentials - Re-enter After Change</t>
+          <t>User Details - Block/Unblock Toggle</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Previously logged in, credentials changed</t>
+          <t>User details panel open</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Verify credentials screen works after clearing credentials</t>
+          <t>Verify Block/Unblock text toggles correctly</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>1. Login successfully
-2. Change credentials from login screen
-3. Re-enter new credentials
-4. Submit</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>New credentials should be accepted and SDK re-initialized</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>USR_076</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Login - Re-login After Logout</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>User previously logged out</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>Verify login works after logout</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>1. Logout from app
-2. Return to login screen
-3. Login again</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>Login should work normally after logout</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>USR_077</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>User Details - Block/Unblock Toggle</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>User details panel open</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Verify Block/Unblock text toggles correctly</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>1. Block user
 2. Observe action text changes to Unblock
@@ -4647,59 +3628,99 @@
 4. Observe text changes to Block</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Action text should toggle between Block and Unblock correctly</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="9" t="n"/>
+      <c r="B9" s="9" t="n"/>
+      <c r="C9" s="9" t="n"/>
+      <c r="D9" s="9" t="n"/>
+      <c r="E9" s="9" t="n"/>
+      <c r="F9" s="9" t="n"/>
+      <c r="G9" s="9" t="n"/>
+      <c r="H9" s="9" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>USR_020</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Unblock After App Restart</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>User unblocked then app restarted</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Verify unblock persists after restart</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>1. Unblock user
 2. Restart app</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>User still unblocked</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="n"/>
+      <c r="B11" s="7" t="n"/>
+      <c r="C11" s="7" t="n"/>
+      <c r="D11" s="7" t="n"/>
+      <c r="E11" s="7" t="n"/>
+      <c r="F11" s="7" t="n"/>
+      <c r="G11" s="7" t="n"/>
+      <c r="H11" s="7" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="n"/>
+      <c r="B12" s="8" t="n"/>
+      <c r="C12" s="8" t="n"/>
+      <c r="D12" s="8" t="n"/>
+      <c r="E12" s="8" t="n"/>
+      <c r="F12" s="8" t="n"/>
+      <c r="G12" s="8" t="n"/>
+      <c r="H12" s="8" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="n"/>
+      <c r="B13" s="7" t="n"/>
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="7" t="n"/>
+      <c r="E13" s="7" t="n"/>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="7" t="n"/>
+      <c r="H13" s="7" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4713,7 +3734,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4875,62 +3896,61 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>USR_078</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Credentials - Auth Key Not Masked</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Credentials screen displayed</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Verify Auth Key input is plain text type</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>1. Enter Auth Key
-2. Observe input type</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Auth Key field uses type='text' (visible for dev convenience)</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
+      <c r="A5" s="8" t="n"/>
+      <c r="B5" s="8" t="n"/>
+      <c r="C5" s="8" t="n"/>
+      <c r="D5" s="8" t="n"/>
+      <c r="E5" s="8" t="n"/>
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="8" t="n"/>
+      <c r="H5" s="8" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="n"/>
-      <c r="B6" s="6" t="n"/>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="6" t="n"/>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="n"/>
-      <c r="H6" s="6" t="n"/>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>USERS_032</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Security: User Module</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>User is not logged in</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Verify user list not accessible without authentication</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>1. Try to access user list without logging in.</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Should redirect to login. No user data exposed.</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>High / Critical</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>USERS_032</t>
+          <t>USR_022</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -4940,248 +3960,94 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Security: User Module</t>
+          <t>Block Bypass via API</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>User is not logged in</t>
+          <t>Direct API call</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Verify user list not accessible without authentication</t>
+          <t>Verify block cannot be bypassed</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>1. Try to access user list without logging in.</t>
+          <t>1. Try to message blocked user via API</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Should redirect to login. No user data exposed.</t>
+          <t>Message rejected for blocked user</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>High / Critical</t>
+          <t>Critical</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>USR_022</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Block Bypass via API</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Direct API call</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Verify block cannot be bypassed</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>1. Try to message blocked user via API</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>Message rejected for blocked user</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
+      <c r="A8" s="8" t="n"/>
+      <c r="B8" s="8" t="n"/>
+      <c r="C8" s="8" t="n"/>
+      <c r="D8" s="8" t="n"/>
+      <c r="E8" s="8" t="n"/>
+      <c r="F8" s="8" t="n"/>
+      <c r="G8" s="8" t="n"/>
+      <c r="H8" s="8" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>USR_079</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Credentials - XSS in App ID</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Credentials screen displayed</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Verify XSS injection in App ID is handled</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>1. Enter &lt;script&gt;alert('xss')&lt;/script&gt; as App ID
-2. Click Continue</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Script should not execute, input treated as plain text</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
+      <c r="A9" s="8" t="n"/>
+      <c r="B9" s="8" t="n"/>
+      <c r="C9" s="8" t="n"/>
+      <c r="D9" s="8" t="n"/>
+      <c r="E9" s="8" t="n"/>
+      <c r="F9" s="8" t="n"/>
+      <c r="G9" s="8" t="n"/>
+      <c r="H9" s="8" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>USR_080</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Credentials - XSS in Auth Key</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Credentials screen displayed</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Verify XSS injection in Auth Key is handled</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>1. Enter &lt;script&gt;alert('xss')&lt;/script&gt; as Auth Key
-2. Click Continue</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>Script should not execute, input treated as plain text</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
+      <c r="A10" s="8" t="n"/>
+      <c r="B10" s="8" t="n"/>
+      <c r="C10" s="8" t="n"/>
+      <c r="D10" s="8" t="n"/>
+      <c r="E10" s="8" t="n"/>
+      <c r="F10" s="8" t="n"/>
+      <c r="G10" s="8" t="n"/>
+      <c r="H10" s="8" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>USR_081</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Login - XSS in Custom UID</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Login screen displayed</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Verify XSS injection in UID field</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>1. Enter &lt;script&gt;alert('xss')&lt;/script&gt; as UID
-2. Click Login</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Script should not execute, treated as plain text UID</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
+      <c r="A11" s="8" t="n"/>
+      <c r="B11" s="8" t="n"/>
+      <c r="C11" s="8" t="n"/>
+      <c r="D11" s="8" t="n"/>
+      <c r="E11" s="8" t="n"/>
+      <c r="F11" s="8" t="n"/>
+      <c r="G11" s="8" t="n"/>
+      <c r="H11" s="8" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>USR_082</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Login - SQL Injection in UID</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Login screen displayed</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Verify SQL injection in UID field</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>1. Enter ' OR 1=1 -- as UID
-2. Click Login</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>Input should be treated as literal string, no injection</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
+      <c r="A12" s="8" t="n"/>
+      <c r="B12" s="8" t="n"/>
+      <c r="C12" s="8" t="n"/>
+      <c r="D12" s="8" t="n"/>
+      <c r="E12" s="8" t="n"/>
+      <c r="F12" s="8" t="n"/>
+      <c r="G12" s="8" t="n"/>
+      <c r="H12" s="8" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="n"/>
+      <c r="B13" s="7" t="n"/>
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="7" t="n"/>
+      <c r="E13" s="7" t="n"/>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="7" t="n"/>
+      <c r="H13" s="7" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5195,7 +4061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5470,7 +4336,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>USR_083</t>
+          <t>USR_085</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -5480,253 +4346,163 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Credentials - Rapid Region Switching</t>
+          <t>User Details - Rapid Block/Unblock</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Credentials screen displayed</t>
+          <t>User details panel open</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Verify rapid switching between regions</t>
+          <t>Verify rapid block/unblock doesn't cause issues</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>1. Click US, then EU, then IN rapidly
-2. Observe final state</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>Only the last clicked region should be selected</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>USR_084</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Login - Rapid Multiple User Clicks</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Sample users displayed</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>Verify rapid clicking different sample users</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>1. Click user A
-2. Immediately click user B
-3. Observe behavior</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>Only one login attempt should proceed, no race condition</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>USR_085</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>User Details - Rapid Block/Unblock</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>User details panel open</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>Verify rapid block/unblock doesn't cause issues</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>1. Block user
 2. Immediately unblock
 3. Repeat rapidly</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Each action should complete before next, no race conditions</t>
         </is>
       </c>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="7" t="n"/>
-      <c r="B11" s="7" t="n"/>
-      <c r="C11" s="7" t="n"/>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
-      <c r="F11" s="7" t="n"/>
-      <c r="G11" s="7" t="n"/>
-      <c r="H11" s="7" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="9" t="n"/>
+      <c r="B9" s="9" t="n"/>
+      <c r="C9" s="9" t="n"/>
+      <c r="D9" s="9" t="n"/>
+      <c r="E9" s="9" t="n"/>
+      <c r="F9" s="9" t="n"/>
+      <c r="G9" s="9" t="n"/>
+      <c r="H9" s="9" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>USERS_039</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="C12" s="2" t="n"/>
-      <c r="D12" s="2" t="n"/>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="C10" s="5" t="n"/>
+      <c r="D10" s="5" t="n"/>
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>Verify user list when server returns error</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>1. Simulate server error.
 2. Open users tab.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>Error message should display with retry option. No crash.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>High / High</t>
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>USR_025</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Block Offline User</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Target user is offline</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Verify can block offline user</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>1. Block an offline user</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>User blocked regardless of online status</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="n"/>
+      <c r="B12" s="8" t="n"/>
+      <c r="C12" s="8" t="n"/>
+      <c r="D12" s="8" t="n"/>
+      <c r="E12" s="8" t="n"/>
+      <c r="F12" s="8" t="n"/>
+      <c r="G12" s="8" t="n"/>
+      <c r="H12" s="8" t="n"/>
+    </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>USR_025</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Block Offline User</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Target user is offline</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Verify can block offline user</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>1. Block an offline user</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>User blocked regardless of online status</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
+      <c r="A13" s="8" t="n"/>
+      <c r="B13" s="8" t="n"/>
+      <c r="C13" s="8" t="n"/>
+      <c r="D13" s="8" t="n"/>
+      <c r="E13" s="8" t="n"/>
+      <c r="F13" s="8" t="n"/>
+      <c r="G13" s="8" t="n"/>
+      <c r="H13" s="8" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>USR_086</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Credentials - Very Long App ID</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Credentials screen displayed</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Verify handling of extremely long App ID</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>1. Enter 1000+ character string as App ID
-2. Click Continue</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>App should handle gracefully, SDK init should fail with proper error</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
+      <c r="A14" s="8" t="n"/>
+      <c r="B14" s="8" t="n"/>
+      <c r="C14" s="8" t="n"/>
+      <c r="D14" s="8" t="n"/>
+      <c r="E14" s="8" t="n"/>
+      <c r="F14" s="8" t="n"/>
+      <c r="G14" s="8" t="n"/>
+      <c r="H14" s="8" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="n"/>
+      <c r="B15" s="7" t="n"/>
+      <c r="C15" s="7" t="n"/>
+      <c r="D15" s="7" t="n"/>
+      <c r="E15" s="7" t="n"/>
+      <c r="F15" s="7" t="n"/>
+      <c r="G15" s="7" t="n"/>
+      <c r="H15" s="7" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5740,7 +4516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5940,84 +4716,49 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>USR_087</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Credentials - Minimum Valid App ID</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Credentials screen displayed</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Verify minimum length App ID (1 char)</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>1. Enter single character as App ID
-2. Enter valid Auth Key
-3. Submit</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Form should submit (HTML validation passes), SDK may reject</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
+      <c r="A6" s="8" t="n"/>
+      <c r="B6" s="8" t="n"/>
+      <c r="C6" s="8" t="n"/>
+      <c r="D6" s="8" t="n"/>
+      <c r="E6" s="8" t="n"/>
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="8" t="n"/>
+      <c r="H6" s="8" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>USR_088</t>
+          <t>USR_027</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Login - Single Character UID</t>
+          <t>Empty Users List</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Login screen displayed</t>
+          <t>No users available</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Verify login with 1-character UID</t>
+          <t>Verify empty state with 0 users</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>1. Enter single character UID
-2. Click Login</t>
+          <t>1. No users in app</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Login attempt should be made with the single character UID</t>
+          <t>Empty state displayed</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -6037,89 +4778,34 @@
       <c r="H8" s="7" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>USR_027</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Empty Users List</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>No users available</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Verify empty state with 0 users</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>1. No users in app</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Empty state displayed</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
+      <c r="A9" s="8" t="n"/>
+      <c r="B9" s="8" t="n"/>
+      <c r="C9" s="8" t="n"/>
+      <c r="D9" s="8" t="n"/>
+      <c r="E9" s="8" t="n"/>
+      <c r="F9" s="8" t="n"/>
+      <c r="G9" s="8" t="n"/>
+      <c r="H9" s="8" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>USR_089</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Login - Very Long UID</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Login screen displayed</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Verify login with extremely long UID (500+ chars)</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>1. Enter 500+ character UID
-2. Click Login</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>Should handle gracefully, SDK should reject or timeout</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
+      <c r="A10" s="8" t="n"/>
+      <c r="B10" s="8" t="n"/>
+      <c r="C10" s="8" t="n"/>
+      <c r="D10" s="8" t="n"/>
+      <c r="E10" s="8" t="n"/>
+      <c r="F10" s="8" t="n"/>
+      <c r="G10" s="8" t="n"/>
+      <c r="H10" s="8" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="n"/>
+      <c r="B11" s="7" t="n"/>
+      <c r="C11" s="7" t="n"/>
+      <c r="D11" s="7" t="n"/>
+      <c r="E11" s="7" t="n"/>
+      <c r="F11" s="7" t="n"/>
+      <c r="G11" s="7" t="n"/>
+      <c r="H11" s="7" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6133,7 +4819,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6375,84 +5061,49 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>USR_090</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Credentials - Valid Hex App ID</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Credentials screen displayed</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Verify valid hexadecimal App ID format</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>1. Enter valid hex string App ID
-2. Enter valid Auth Key
-3. Submit</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Credentials should be accepted and SDK initialized</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
+      <c r="A7" s="8" t="n"/>
+      <c r="B7" s="8" t="n"/>
+      <c r="C7" s="8" t="n"/>
+      <c r="D7" s="8" t="n"/>
+      <c r="E7" s="8" t="n"/>
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="8" t="n"/>
+      <c r="H7" s="8" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>USR_091</t>
+          <t>USR_030</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Login - Alphanumeric UID</t>
+          <t>Blocked User</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Login screen displayed</t>
+          <t>User is blocked</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Verify login with alphanumeric UID</t>
+          <t>Verify blocked user display</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>1. Enter UID like 'user123'
-2. Click Login</t>
+          <t>1. Check blocked user in list</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Login should proceed normally</t>
+          <t>Blocked indicator or different styling shown</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -6472,132 +5123,44 @@
       <c r="H9" s="7" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>USR_030</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Blocked User</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>User is blocked</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Verify blocked user display</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>1. Check blocked user in list</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>Blocked indicator or different styling shown</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
+      <c r="A10" s="8" t="n"/>
+      <c r="B10" s="8" t="n"/>
+      <c r="C10" s="8" t="n"/>
+      <c r="D10" s="8" t="n"/>
+      <c r="E10" s="8" t="n"/>
+      <c r="F10" s="8" t="n"/>
+      <c r="G10" s="8" t="n"/>
+      <c r="H10" s="8" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>USR_092</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Credentials - Special Chars in App ID</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Credentials screen displayed</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Verify special characters in App ID</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>1. Enter App ID with special chars (!@#$%)
-2. Submit</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>SDK should reject invalid App ID format</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
+      <c r="A11" s="8" t="n"/>
+      <c r="B11" s="8" t="n"/>
+      <c r="C11" s="8" t="n"/>
+      <c r="D11" s="8" t="n"/>
+      <c r="E11" s="8" t="n"/>
+      <c r="F11" s="8" t="n"/>
+      <c r="G11" s="8" t="n"/>
+      <c r="H11" s="8" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>USR_093</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Login - UID with Spaces</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Login screen displayed</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Verify login with UID containing spaces</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>1. Enter 'user 123' as UID
-2. Click Login</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>SDK should handle or reject UID with spaces</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
+      <c r="A12" s="8" t="n"/>
+      <c r="B12" s="8" t="n"/>
+      <c r="C12" s="8" t="n"/>
+      <c r="D12" s="8" t="n"/>
+      <c r="E12" s="8" t="n"/>
+      <c r="F12" s="8" t="n"/>
+      <c r="G12" s="8" t="n"/>
+      <c r="H12" s="8" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="n"/>
+      <c r="B13" s="7" t="n"/>
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="7" t="n"/>
+      <c r="E13" s="7" t="n"/>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="7" t="n"/>
+      <c r="H13" s="7" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>